<commit_message>
feat(member): enrich service and fault records
</commit_message>
<xml_diff>
--- a/public/downloads/sample-ipace-owner-data.xlsx
+++ b/public/downloads/sample-ipace-owner-data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>My I-PACE owner data</t>
   </si>
@@ -239,6 +239,15 @@
     <t>Campaigns</t>
   </si>
   <si>
+    <t>Service provider</t>
+  </si>
+  <si>
+    <t>Provider postcode</t>
+  </si>
+  <si>
+    <t>Authorised JLR provider</t>
+  </si>
+  <si>
     <t>Final fix date</t>
   </si>
   <si>
@@ -254,6 +263,12 @@
     <t>Parts delay</t>
   </si>
   <si>
+    <t>Goodwill payment</t>
+  </si>
+  <si>
+    <t>Miles driven whilst faulty</t>
+  </si>
+  <si>
     <t>Warranty cover</t>
   </si>
   <si>
@@ -275,49 +290,67 @@
     <t>Sample campaign A</t>
   </si>
   <si>
+    <t>Example Jaguar North</t>
+  </si>
+  <si>
+    <t>AB1 2CD</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>2025-11-20</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>up-to-1-week</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>2026-03-08</t>
+  </si>
+  <si>
+    <t>Scheduled service</t>
+  </si>
+  <si>
+    <t>Routine inspection and software updates.</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>2026-02-11</t>
+  </si>
+  <si>
+    <t>Recall inspection</t>
+  </si>
+  <si>
+    <t>Vehicle inspected and returned the same day.</t>
+  </si>
+  <si>
+    <t>Sample campaign B</t>
+  </si>
+  <si>
+    <t>Example Jaguar South</t>
+  </si>
+  <si>
+    <t>XY9 8ZZ</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Full</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>2026-03-08</t>
-  </si>
-  <si>
-    <t>Scheduled service</t>
-  </si>
-  <si>
-    <t>Routine inspection and software updates.</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>2026-02-11</t>
-  </si>
-  <si>
-    <t>Recall inspection</t>
-  </si>
-  <si>
-    <t>Vehicle inspected and returned the same day.</t>
-  </si>
-  <si>
-    <t>Sample campaign B</t>
+    <t>none</t>
   </si>
   <si>
     <t>Battery health check</t>
@@ -984,9 +1017,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ServiceAndFaultsTable" displayName="ServiceAndFaultsTable" ref="A1:Q5">
-  <autoFilter ref="A1:Q5"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ServiceAndFaultsTable" displayName="ServiceAndFaultsTable" ref="A1:V5">
+  <autoFilter ref="A1:V5"/>
+  <tableColumns count="22">
     <tableColumn id="1" name="Vehicle"/>
     <tableColumn id="2" name="Type"/>
     <tableColumn id="3" name="Date"/>
@@ -995,15 +1028,20 @@
     <tableColumn id="6" name="Description"/>
     <tableColumn id="7" name="Status"/>
     <tableColumn id="8" name="Campaigns"/>
-    <tableColumn id="9" name="Final fix date"/>
-    <tableColumn id="10" name="Days to final fix"/>
-    <tableColumn id="11" name="Courtesy vehicle offered"/>
-    <tableColumn id="12" name="Courtesy vehicle provided"/>
-    <tableColumn id="13" name="Parts delay"/>
-    <tableColumn id="14" name="Warranty cover"/>
-    <tableColumn id="15" name="Dispute status"/>
-    <tableColumn id="16" name="Created"/>
-    <tableColumn id="17" name="Updated"/>
+    <tableColumn id="9" name="Service provider"/>
+    <tableColumn id="10" name="Provider postcode"/>
+    <tableColumn id="11" name="Authorised JLR provider"/>
+    <tableColumn id="12" name="Final fix date"/>
+    <tableColumn id="13" name="Days to final fix"/>
+    <tableColumn id="14" name="Courtesy vehicle offered"/>
+    <tableColumn id="15" name="Courtesy vehicle provided"/>
+    <tableColumn id="16" name="Parts delay"/>
+    <tableColumn id="17" name="Goodwill payment"/>
+    <tableColumn id="18" name="Miles driven whilst faulty"/>
+    <tableColumn id="19" name="Warranty cover"/>
+    <tableColumn id="20" name="Dispute status"/>
+    <tableColumn id="21" name="Created"/>
+    <tableColumn id="22" name="Updated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
 </table>
@@ -1772,7 +1810,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="17" min="1" width="18"/>
+    <col customWidth="true" max="22" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
@@ -1822,9 +1860,24 @@
         <v>79</v>
       </c>
       <c r="P1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1836,48 +1889,63 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D2">
         <v>40230</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
-      </c>
-      <c r="J2">
+        <v>90</v>
+      </c>
+      <c r="J2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" t="s">
+        <v>93</v>
+      </c>
+      <c r="M2">
         <v>6</v>
       </c>
-      <c r="K2" t="s">
-        <v>86</v>
-      </c>
-      <c r="L2" t="s">
-        <v>86</v>
-      </c>
-      <c r="M2" t="s">
-        <v>87</v>
-      </c>
       <c r="N2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="O2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="P2" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>92</v>
+      </c>
+      <c r="R2">
+        <v>220</v>
+      </c>
+      <c r="S2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T2" t="s">
+        <v>96</v>
+      </c>
+      <c r="U2" t="s">
         <v>51</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="V2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1889,48 +1957,63 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D3">
         <v>44700</v>
       </c>
       <c r="E3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J3" t="s">
         <v>91</v>
       </c>
-      <c r="F3" t="s">
+      <c r="K3" t="s">
         <v>92</v>
       </c>
-      <c r="G3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" t="s">
-        <v>94</v>
-      </c>
-      <c r="J3" t="s">
-        <v>94</v>
-      </c>
-      <c r="K3" t="s">
-        <v>94</v>
-      </c>
       <c r="L3" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="M3" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O3" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="P3" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>101</v>
+      </c>
+      <c r="R3" t="s">
+        <v>101</v>
+      </c>
+      <c r="S3" t="s">
+        <v>102</v>
+      </c>
+      <c r="T3" t="s">
+        <v>96</v>
+      </c>
+      <c r="U3" t="s">
         <v>51</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="V3" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1942,48 +2025,63 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D4">
         <v>17540</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="I4" t="s">
+        <v>107</v>
+      </c>
+      <c r="J4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" t="s">
+        <v>103</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="s">
+        <v>109</v>
+      </c>
+      <c r="O4" t="s">
+        <v>109</v>
+      </c>
+      <c r="P4" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
+        <v>95</v>
+      </c>
+      <c r="T4" t="s">
         <v>96</v>
       </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" t="s">
-        <v>87</v>
-      </c>
-      <c r="M4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N4" t="s">
-        <v>88</v>
-      </c>
-      <c r="O4" t="s">
-        <v>89</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="U4" t="s">
         <v>51</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="V4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2001,42 +2099,57 @@
         <v>21790</v>
       </c>
       <c r="E5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" t="s">
         <v>100</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>101</v>
       </c>
-      <c r="G5" t="s">
-        <v>93</v>
-      </c>
-      <c r="H5" t="s">
-        <v>94</v>
-      </c>
       <c r="I5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="J5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="K5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="L5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O5" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="P5" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>101</v>
+      </c>
+      <c r="R5" t="s">
+        <v>101</v>
+      </c>
+      <c r="S5" t="s">
+        <v>102</v>
+      </c>
+      <c r="T5" t="s">
+        <v>96</v>
+      </c>
+      <c r="U5" t="s">
         <v>51</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="V5" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(member): enrich service and fault records (#82)
</commit_message>
<xml_diff>
--- a/public/downloads/sample-ipace-owner-data.xlsx
+++ b/public/downloads/sample-ipace-owner-data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>My I-PACE owner data</t>
   </si>
@@ -239,6 +239,15 @@
     <t>Campaigns</t>
   </si>
   <si>
+    <t>Service provider</t>
+  </si>
+  <si>
+    <t>Provider postcode</t>
+  </si>
+  <si>
+    <t>Authorised JLR provider</t>
+  </si>
+  <si>
     <t>Final fix date</t>
   </si>
   <si>
@@ -254,6 +263,12 @@
     <t>Parts delay</t>
   </si>
   <si>
+    <t>Goodwill payment</t>
+  </si>
+  <si>
+    <t>Miles driven whilst faulty</t>
+  </si>
+  <si>
     <t>Warranty cover</t>
   </si>
   <si>
@@ -275,49 +290,67 @@
     <t>Sample campaign A</t>
   </si>
   <si>
+    <t>Example Jaguar North</t>
+  </si>
+  <si>
+    <t>AB1 2CD</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>2025-11-20</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>up-to-1-week</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>2026-03-08</t>
+  </si>
+  <si>
+    <t>Scheduled service</t>
+  </si>
+  <si>
+    <t>Routine inspection and software updates.</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>2026-02-11</t>
+  </si>
+  <si>
+    <t>Recall inspection</t>
+  </si>
+  <si>
+    <t>Vehicle inspected and returned the same day.</t>
+  </si>
+  <si>
+    <t>Sample campaign B</t>
+  </si>
+  <si>
+    <t>Example Jaguar South</t>
+  </si>
+  <si>
+    <t>XY9 8ZZ</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Full</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>2026-03-08</t>
-  </si>
-  <si>
-    <t>Scheduled service</t>
-  </si>
-  <si>
-    <t>Routine inspection and software updates.</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>2026-02-11</t>
-  </si>
-  <si>
-    <t>Recall inspection</t>
-  </si>
-  <si>
-    <t>Vehicle inspected and returned the same day.</t>
-  </si>
-  <si>
-    <t>Sample campaign B</t>
+    <t>none</t>
   </si>
   <si>
     <t>Battery health check</t>
@@ -984,9 +1017,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ServiceAndFaultsTable" displayName="ServiceAndFaultsTable" ref="A1:Q5">
-  <autoFilter ref="A1:Q5"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ServiceAndFaultsTable" displayName="ServiceAndFaultsTable" ref="A1:V5">
+  <autoFilter ref="A1:V5"/>
+  <tableColumns count="22">
     <tableColumn id="1" name="Vehicle"/>
     <tableColumn id="2" name="Type"/>
     <tableColumn id="3" name="Date"/>
@@ -995,15 +1028,20 @@
     <tableColumn id="6" name="Description"/>
     <tableColumn id="7" name="Status"/>
     <tableColumn id="8" name="Campaigns"/>
-    <tableColumn id="9" name="Final fix date"/>
-    <tableColumn id="10" name="Days to final fix"/>
-    <tableColumn id="11" name="Courtesy vehicle offered"/>
-    <tableColumn id="12" name="Courtesy vehicle provided"/>
-    <tableColumn id="13" name="Parts delay"/>
-    <tableColumn id="14" name="Warranty cover"/>
-    <tableColumn id="15" name="Dispute status"/>
-    <tableColumn id="16" name="Created"/>
-    <tableColumn id="17" name="Updated"/>
+    <tableColumn id="9" name="Service provider"/>
+    <tableColumn id="10" name="Provider postcode"/>
+    <tableColumn id="11" name="Authorised JLR provider"/>
+    <tableColumn id="12" name="Final fix date"/>
+    <tableColumn id="13" name="Days to final fix"/>
+    <tableColumn id="14" name="Courtesy vehicle offered"/>
+    <tableColumn id="15" name="Courtesy vehicle provided"/>
+    <tableColumn id="16" name="Parts delay"/>
+    <tableColumn id="17" name="Goodwill payment"/>
+    <tableColumn id="18" name="Miles driven whilst faulty"/>
+    <tableColumn id="19" name="Warranty cover"/>
+    <tableColumn id="20" name="Dispute status"/>
+    <tableColumn id="21" name="Created"/>
+    <tableColumn id="22" name="Updated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
 </table>
@@ -1772,7 +1810,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="17" min="1" width="18"/>
+    <col customWidth="true" max="22" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
@@ -1822,9 +1860,24 @@
         <v>79</v>
       </c>
       <c r="P1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1836,48 +1889,63 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D2">
         <v>40230</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
-      </c>
-      <c r="J2">
+        <v>90</v>
+      </c>
+      <c r="J2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" t="s">
+        <v>93</v>
+      </c>
+      <c r="M2">
         <v>6</v>
       </c>
-      <c r="K2" t="s">
-        <v>86</v>
-      </c>
-      <c r="L2" t="s">
-        <v>86</v>
-      </c>
-      <c r="M2" t="s">
-        <v>87</v>
-      </c>
       <c r="N2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="O2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="P2" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>92</v>
+      </c>
+      <c r="R2">
+        <v>220</v>
+      </c>
+      <c r="S2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T2" t="s">
+        <v>96</v>
+      </c>
+      <c r="U2" t="s">
         <v>51</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="V2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1889,48 +1957,63 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D3">
         <v>44700</v>
       </c>
       <c r="E3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J3" t="s">
         <v>91</v>
       </c>
-      <c r="F3" t="s">
+      <c r="K3" t="s">
         <v>92</v>
       </c>
-      <c r="G3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" t="s">
-        <v>94</v>
-      </c>
-      <c r="J3" t="s">
-        <v>94</v>
-      </c>
-      <c r="K3" t="s">
-        <v>94</v>
-      </c>
       <c r="L3" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="M3" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O3" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="P3" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>101</v>
+      </c>
+      <c r="R3" t="s">
+        <v>101</v>
+      </c>
+      <c r="S3" t="s">
+        <v>102</v>
+      </c>
+      <c r="T3" t="s">
+        <v>96</v>
+      </c>
+      <c r="U3" t="s">
         <v>51</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="V3" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1942,48 +2025,63 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D4">
         <v>17540</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="I4" t="s">
+        <v>107</v>
+      </c>
+      <c r="J4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" t="s">
+        <v>103</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="s">
+        <v>109</v>
+      </c>
+      <c r="O4" t="s">
+        <v>109</v>
+      </c>
+      <c r="P4" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
+        <v>95</v>
+      </c>
+      <c r="T4" t="s">
         <v>96</v>
       </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" t="s">
-        <v>87</v>
-      </c>
-      <c r="M4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N4" t="s">
-        <v>88</v>
-      </c>
-      <c r="O4" t="s">
-        <v>89</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="U4" t="s">
         <v>51</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="V4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2001,42 +2099,57 @@
         <v>21790</v>
       </c>
       <c r="E5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" t="s">
         <v>100</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>101</v>
       </c>
-      <c r="G5" t="s">
-        <v>93</v>
-      </c>
-      <c r="H5" t="s">
-        <v>94</v>
-      </c>
       <c r="I5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="J5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="K5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="L5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O5" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="P5" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>101</v>
+      </c>
+      <c r="R5" t="s">
+        <v>101</v>
+      </c>
+      <c r="S5" t="s">
+        <v>102</v>
+      </c>
+      <c r="T5" t="s">
+        <v>96</v>
+      </c>
+      <c r="U5" t="s">
         <v>51</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="V5" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>